<commit_message>
calibration_redux.m polished for plots and comps
</commit_message>
<xml_diff>
--- a/output/med_shocks_redux_popbetas.xlsx
+++ b/output/med_shocks_redux_popbetas.xlsx
@@ -13,7 +13,391 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
   <si>
     <t>med_Q_2</t>
   </si>
@@ -129,7 +513,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -138,13 +522,21 @@
       <diagonal/>
     </border>
     <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -202,7 +594,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="B1" s="0">
         <v>-60.354500143052931</v>
@@ -327,7 +719,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>129</v>
       </c>
       <c r="B2" s="0">
         <v>-62.09682088184374</v>
@@ -452,7 +844,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>130</v>
       </c>
       <c r="B3" s="0">
         <v>-64.927063193970014</v>
@@ -577,7 +969,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="B4" s="0">
         <v>-66.479353419153767</v>
@@ -702,7 +1094,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>4</v>
+        <v>132</v>
       </c>
       <c r="B5" s="0">
         <v>-68.112276544340489</v>
@@ -827,7 +1219,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>5</v>
+        <v>133</v>
       </c>
       <c r="B6" s="0">
         <v>-71.866303085731261</v>
@@ -952,7 +1344,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>6</v>
+        <v>134</v>
       </c>
       <c r="B7" s="0">
         <v>-75.76292724401857</v>
@@ -1077,7 +1469,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>7</v>
+        <v>135</v>
       </c>
       <c r="B8" s="0">
         <v>-77.939170114890629</v>
@@ -1202,7 +1594,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>8</v>
+        <v>136</v>
       </c>
       <c r="B9" s="0">
         <v>-78.792794945987197</v>
@@ -1327,7 +1719,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>9</v>
+        <v>137</v>
       </c>
       <c r="B10" s="0">
         <v>-78.78048511430373</v>
@@ -1452,7 +1844,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>10</v>
+        <v>138</v>
       </c>
       <c r="B11" s="0">
         <v>-78.020552001811154</v>
@@ -1577,7 +1969,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>11</v>
+        <v>139</v>
       </c>
       <c r="B12" s="0">
         <v>-76.945421080172807</v>
@@ -1702,7 +2094,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>12</v>
+        <v>140</v>
       </c>
       <c r="B13" s="0">
         <v>-75.635961403310148</v>
@@ -1827,7 +2219,7 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
       <c r="B14" s="0">
         <v>-74.229566105226198</v>
@@ -1952,7 +2344,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>14</v>
+        <v>142</v>
       </c>
       <c r="B15" s="0">
         <v>-72.794086202841314</v>
@@ -2077,7 +2469,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>15</v>
+        <v>143</v>
       </c>
       <c r="B16" s="0">
         <v>-71.347640780407943</v>
@@ -2202,7 +2594,7 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>16</v>
+        <v>144</v>
       </c>
       <c r="B17" s="0">
         <v>-81.473532862879907</v>
@@ -2327,7 +2719,7 @@
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="B18" s="0">
         <v>-81.416011979970989</v>
@@ -2452,7 +2844,7 @@
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>18</v>
+        <v>146</v>
       </c>
       <c r="B19" s="0">
         <v>-80.637259733084534</v>
@@ -2577,7 +2969,7 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>19</v>
+        <v>147</v>
       </c>
       <c r="B20" s="0">
         <v>-80.211442461834466</v>
@@ -2702,7 +3094,7 @@
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="B21" s="0">
         <v>-79.841542077356451</v>
@@ -2827,7 +3219,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>21</v>
+        <v>149</v>
       </c>
       <c r="B22" s="0">
         <v>-80.003647896245525</v>
@@ -2952,7 +3344,7 @@
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="B23" s="0">
         <v>-80.425429765766751</v>
@@ -3077,7 +3469,7 @@
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>23</v>
+        <v>151</v>
       </c>
       <c r="B24" s="0">
         <v>-80.423700406908281</v>
@@ -3202,7 +3594,7 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>24</v>
+        <v>152</v>
       </c>
       <c r="B25" s="0">
         <v>-80.028050398547421</v>
@@ -3327,7 +3719,7 @@
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>25</v>
+        <v>153</v>
       </c>
       <c r="B26" s="0">
         <v>-79.314296726293904</v>
@@ -3452,7 +3844,7 @@
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>26</v>
+        <v>154</v>
       </c>
       <c r="B27" s="0">
         <v>-78.306812487952882</v>
@@ -3577,7 +3969,7 @@
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>27</v>
+        <v>155</v>
       </c>
       <c r="B28" s="0">
         <v>-77.085047727086604</v>
@@ -3702,7 +4094,7 @@
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>28</v>
+        <v>156</v>
       </c>
       <c r="B29" s="0">
         <v>-75.704991875877454</v>
@@ -3827,7 +4219,7 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>29</v>
+        <v>157</v>
       </c>
       <c r="B30" s="0">
         <v>-74.263546405287414</v>
@@ -3952,7 +4344,7 @@
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>30</v>
+        <v>158</v>
       </c>
       <c r="B31" s="0">
         <v>-72.809959440762825</v>
@@ -4077,7 +4469,7 @@
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>31</v>
+        <v>159</v>
       </c>
       <c r="B32" s="0">
         <v>-71.355772164107151</v>

</xml_diff>